<commit_message>
feat(F-NAR-016): TREE-DIF-031 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-DIF-031.xlsx
+++ b/stories/arbres/TREE-DIF-031.xlsx
@@ -3897,12 +3897,12 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Nina reste collée à l'ombre du figuier. L'eau, l'ombre des plants, ou plus tard ?</t>
+          <t>Nina reste collée à l'ombre du figuier. L'eau, l'ombre des plants, ou garder une tomate ?</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Nina reste collée à l'ombre du figuier. L'eau, l'ombre des plants, ou plus tard ?</t>
+          <t>Nina reste collée à l'ombre du figuier. L'eau, l'ombre des plants, ou garder une tomate ?</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -4062,7 +4062,7 @@
       <c r="AW17" t="inlineStr">
         <is>
           <t>narrateur|Nina reste collée à l'ombre du figuier.
-maman|L'eau, l'ombre des plants, ou plus tard ?</t>
+maman|L'eau, l'ombre des plants, ou garder une tomate ?</t>
         </is>
       </c>
     </row>
@@ -8185,12 +8185,12 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Le caillou blanc veille entre les tomates. Tu as dit oui, avec lui. Il a tout vu, du panier. Vous avez cueilli sans tirer. Goûtez un peu, tout doux. Le chapeau de paille sèche sur la marche. Nina croque, le jus lui tache le menton. Reste autant que tu veux. Le sel brille déjà sur la marche.</t>
+          <t>Le caillou blanc veille entre les tomates. Tu as dit oui, avec lui. Il a tout vu, du chapeau. Vous avez cueilli sans tirer. Goûtez un peu, tout doux. Le chapeau de paille sèche sur la marche. Nina croque, le jus lui tache le menton. Reste autant que tu veux. Le sel brille déjà sur la marche.</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Le caillou blanc veille entre les tomates. Tu as dit oui, avec lui. Il a tout vu, du panier. Vous avez cueilli sans tirer. Goûtez un peu, tout doux. Le chapeau de paille sèche sur la marche. Nina croque, le jus lui tache le menton. Reste autant que tu veux. Le sel brille déjà sur la marche.</t>
+          <t>Le caillou blanc veille entre les tomates. Tu as dit oui, avec lui. Il a tout vu, du chapeau. Vous avez cueilli sans tirer. Goûtez un peu, tout doux. Le chapeau de paille sèche sur la marche. Nina croque, le jus lui tache le menton. Reste autant que tu veux. Le sel brille déjà sur la marche.</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -8327,7 +8327,7 @@
         <is>
           <t>narrateur|Le caillou blanc veille entre les tomates.
 enfant-m|Tu as dit oui, avec lui.
-copine|Il a tout vu, du panier.
+copine|Il a tout vu, du chapeau.
 papa|Vous avez cueilli sans tirer.
 maman|Goûtez un peu, tout doux.
 narrateur|Le chapeau de paille sèche sur la marche.
@@ -8885,12 +8885,12 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Nina reste collée à l'ombre du figuier. L'eau, l'ombre des plants, ou plus tard ?</t>
+          <t>Nina reste collée à l'ombre du figuier. L'eau, l'ombre des plants, ou garder une tomate ?</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>Nina reste collée à l'ombre du figuier. L'eau, l'ombre des plants, ou plus tard ?</t>
+          <t>Nina reste collée à l'ombre du figuier. L'eau, l'ombre des plants, ou garder une tomate ?</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -9050,7 +9050,7 @@
       <c r="AW45" t="inlineStr">
         <is>
           <t>narrateur|Nina reste collée à l'ombre du figuier.
-maman|L'eau, l'ombre des plants, ou plus tard ?</t>
+maman|L'eau, l'ombre des plants, ou garder une tomate ?</t>
         </is>
       </c>
     </row>
@@ -10127,12 +10127,12 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Le chapeau de paille pose une paille d'ombre sur le bac. Nina patouille un gâteau de sable. Il n'est pas cuit, encore. Les tomates m'attendent. Le gâteau penche, tout mouillé. Tu viens cueillir ? Après, peut-être. Son gâteau n'est pas fini. Tu proposes quoi, Raphaël ?</t>
+          <t>Le chapeau de paille fait un rond sur le bac. Nina patouille un gâteau de sable. Il n'est pas cuit, encore. Les tomates m'attendent. Le gâteau penche, tout mouillé. Tu viens cueillir ? Après, peut-être. Son gâteau n'est pas fini. Tu proposes quoi, Raphaël ?</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Le chapeau de paille pose une paille d'ombre sur le bac. Nina patouille un gâteau de sable. Il n'est pas cuit, encore. Les tomates m'attendent. Le gâteau penche, tout mouillé. Tu viens cueillir ? Après, peut-être. Son gâteau n'est pas fini. Tu proposes quoi, Raphaël ?</t>
+          <t>Le chapeau de paille fait un rond sur le bac. Nina patouille un gâteau de sable. Il n'est pas cuit, encore. Les tomates m'attendent. Le gâteau penche, tout mouillé. Tu viens cueillir ? Après, peut-être. Son gâteau n'est pas fini. Tu proposes quoi, Raphaël ?</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -10267,7 +10267,7 @@
       <c r="AV52" s="2" t="inlineStr"/>
       <c r="AW52" t="inlineStr">
         <is>
-          <t>narrateur|Le chapeau de paille pose une paille d'ombre sur le bac.
+          <t>narrateur|Le chapeau de paille fait un rond sur le bac.
 narrateur|Nina patouille un gâteau de sable.
 copine|Il n'est pas cuit, encore.
 enfant-m|Les tomates m'attendent.
@@ -13173,12 +13173,12 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Le caillou blanc veille entre les tomates. Tu as dit oui, avec lui. Il a tout vu, du panier. Vous avez cueilli sans tirer. Goûtez un peu, tout doux. Le petit tabouret reste près du pain. Nina croque, le jus lui tache le menton. Reste autant que tu veux. Le sel brille déjà sur la marche.</t>
+          <t>Le caillou blanc veille entre les tomates. Tu as dit oui, avec lui. Il a tout vu, du tabouret. Vous avez cueilli sans tirer. Goûtez un peu, tout doux. Le petit tabouret reste près du pain. Nina croque, le jus lui tache le menton. Reste autant que tu veux. Le sel brille déjà sur la marche.</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>Le caillou blanc veille entre les tomates. Tu as dit oui, avec lui. Il a tout vu, du panier. Vous avez cueilli sans tirer. Goûtez un peu, tout doux. Le petit tabouret reste près du pain. Nina croque, le jus lui tache le menton. Reste autant que tu veux. Le sel brille déjà sur la marche.</t>
+          <t>Le caillou blanc veille entre les tomates. Tu as dit oui, avec lui. Il a tout vu, du tabouret. Vous avez cueilli sans tirer. Goûtez un peu, tout doux. Le petit tabouret reste près du pain. Nina croque, le jus lui tache le menton. Reste autant que tu veux. Le sel brille déjà sur la marche.</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -13315,7 +13315,7 @@
         <is>
           <t>narrateur|Le caillou blanc veille entre les tomates.
 enfant-m|Tu as dit oui, avec lui.
-copine|Il a tout vu, du panier.
+copine|Il a tout vu, du tabouret.
 papa|Vous avez cueilli sans tirer.
 maman|Goûtez un peu, tout doux.
 narrateur|Le petit tabouret reste près du pain.
@@ -13873,12 +13873,12 @@
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>Nina reste collée à l'ombre du figuier. L'eau, l'ombre des plants, ou plus tard ?</t>
+          <t>Nina reste collée à l'ombre du figuier. L'eau, l'ombre des plants, ou garder une tomate ?</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>Nina reste collée à l'ombre du figuier. L'eau, l'ombre des plants, ou plus tard ?</t>
+          <t>Nina reste collée à l'ombre du figuier. L'eau, l'ombre des plants, ou garder une tomate ?</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -14038,7 +14038,7 @@
       <c r="AW73" t="inlineStr">
         <is>
           <t>narrateur|Nina reste collée à l'ombre du figuier.
-maman|L'eau, l'ombre des plants, ou plus tard ?</t>
+maman|L'eau, l'ombre des plants, ou garder une tomate ?</t>
         </is>
       </c>
     </row>
@@ -16526,7 +16526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -16576,6 +16576,20 @@
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>